<commit_message>
Corrected one wqreference for ichneumonid traits
</commit_message>
<xml_diff>
--- a/source_data/Ichneumonidae_traits.xlsx
+++ b/source_data/Ichneumonidae_traits.xlsx
@@ -5,10 +5,10 @@
   <workbookPr date1904="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/traits/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C908AF2-A6E3-D943-B355-DFEC852A2DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B26C397-ADC1-BB4D-B103-8CDD445BFE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28140" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -378,7 +378,7 @@
     <t>Phygadeuontinae_s_str</t>
   </si>
   <si>
-    <t>van Achtenberg (2013)</t>
+    <t>van Achtenberg &amp; Altenhofer (2013)</t>
   </si>
 </sst>
 </file>
@@ -823,7 +823,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -867,7 +867,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">

</xml_diff>

<commit_message>
Minor corrections to Ichneumonidae traits data
</commit_message>
<xml_diff>
--- a/source_data/Ichneumonidae_traits.xlsx
+++ b/source_data/Ichneumonidae_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B26C397-ADC1-BB4D-B103-8CDD445BFE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F30A96-D863-5D42-82E9-14022C1A2E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28140" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -366,9 +366,6 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>Ephialtinae_s_str</t>
-  </si>
-  <si>
     <t>Polysphincta_group</t>
   </si>
   <si>
@@ -379,6 +376,9 @@
   </si>
   <si>
     <t>van Achtenberg &amp; Altenhofer (2013)</t>
+  </si>
+  <si>
+    <t>Pimplinae_s_str</t>
   </si>
 </sst>
 </file>
@@ -823,7 +823,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -867,7 +867,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -1509,7 +1509,7 @@
         <v>2</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="13" customHeight="1">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>1</v>
@@ -2047,7 +2047,7 @@
         <v>93</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>1</v>
@@ -2074,7 +2074,7 @@
         <v>59</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>1</v>
@@ -2101,7 +2101,7 @@
         <v>64</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>1</v>
@@ -2128,7 +2128,7 @@
         <v>64</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Resolved last issues based on mail from Seraina 2026-02-11
</commit_message>
<xml_diff>
--- a/source_data/Ichneumonidae_traits.xlsx
+++ b/source_data/Ichneumonidae_traits.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10308"/>
   <workbookPr date1904="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86D9A38-F561-FB44-9FE9-3D18530304C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DFE003E-7008-0F4A-94B8-422EBCEA1F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28140" windowHeight="17460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="620" windowWidth="25400" windowHeight="15400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Swedish data" sheetId="1" r:id="rId1"/>
+    <sheet name="Trait data" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Swedish data'!$B$1:$F$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Trait data'!$B$1:$F$57</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="112">
   <si>
     <t>Saprophage-parasitoid</t>
     <phoneticPr fontId="3"/>
@@ -216,24 +216,12 @@
     <t>Xoridinae</t>
   </si>
   <si>
-    <t>Main feeding niche SE</t>
-  </si>
-  <si>
-    <t>Main feeding habitat SE</t>
-  </si>
-  <si>
     <t>Ateleutinae</t>
   </si>
   <si>
     <t>Nesomesochorinae</t>
   </si>
   <si>
-    <t>Main feeding niche MG</t>
-  </si>
-  <si>
-    <t>Main feeding habitat MG</t>
-  </si>
-  <si>
     <t>Pimplini</t>
   </si>
   <si>
@@ -243,9 +231,6 @@
     <t>Plants</t>
   </si>
   <si>
-    <t>? habitat classification</t>
-  </si>
-  <si>
     <t>Tribe</t>
   </si>
   <si>
@@ -264,9 +249,6 @@
     <t>Gavin R. Broad, unpublished data</t>
   </si>
   <si>
-    <t>? also on saprophagous Coleoptera in soil or wood</t>
-  </si>
-  <si>
     <t>Sisyrostolinae</t>
   </si>
   <si>
@@ -327,15 +309,9 @@
     <t>Labenini</t>
   </si>
   <si>
-    <t>Saprophage-parasitoid</t>
-  </si>
-  <si>
     <t>Wood</t>
   </si>
   <si>
-    <t>Life history?? (suggestion from Wikipedia, and Gauld &amp; Wahl 2008)</t>
-  </si>
-  <si>
     <t>Phygadeuontinae</t>
   </si>
   <si>
@@ -378,14 +354,69 @@
     <t>Pimplinae_s_str</t>
   </si>
   <si>
-    <t>Hybrizoninae</t>
+    <t>The Coleoptera hosts are typically Tenebrionidae on plants</t>
+  </si>
+  <si>
+    <t>Spider parasitoids. Most of the hosts are on vegetation.</t>
+  </si>
+  <si>
+    <t>Hybrizontinae</t>
+  </si>
+  <si>
+    <t>Fungi</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Diacritus aciculatus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> has been reared from a fungus. Host is unknown but assumed here to be a saprophage.</t>
+    </r>
+  </si>
+  <si>
+    <t>Some species have secondarily switched to being predator parasitoids.</t>
+  </si>
+  <si>
+    <t>Gauld &amp; Wahl (2000)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most species attack Lepidoptera cocoons in leaf rolls and in other weakly concealed sites on plants. </t>
+  </si>
+  <si>
+    <t>Ephialtini_Theronini</t>
+  </si>
+  <si>
+    <t>Most species are likely associated with hosts on plants; some species are associated with hosts in wood, which may be the ancestral life history</t>
+  </si>
+  <si>
+    <t>Feeding niche SE</t>
+  </si>
+  <si>
+    <t>Feeding habitat SE</t>
+  </si>
+  <si>
+    <t>Feeding niche MG</t>
+  </si>
+  <si>
+    <t>Feeding habitat MG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -444,25 +475,19 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFD9A"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -477,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -492,8 +517,22 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -893,13 +932,13 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="47.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="2" width="17" style="1" customWidth="1"/>
-    <col min="3" max="3" width="19.1640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.1640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="23.6640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="28.83203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="22.6640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="23.5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="56.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="56.6640625" style="12" customWidth="1"/>
     <col min="10" max="16384" width="47.1640625" style="1"/>
   </cols>
   <sheetData>
@@ -911,25 +950,25 @@
         <v>18</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>56</v>
+        <v>110</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="13" customHeight="1">
@@ -955,7 +994,7 @@
       <c r="H2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="7"/>
+      <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:9" ht="13" customHeight="1">
       <c r="A3" s="7" t="s">
@@ -980,7 +1019,7 @@
       <c r="H3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="7"/>
+      <c r="I3" s="10"/>
     </row>
     <row r="4" spans="1:9" ht="13" customHeight="1">
       <c r="A4" s="7" t="s">
@@ -1005,9 +1044,9 @@
       <c r="H4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" spans="1:9" ht="13" customHeight="1">
+      <c r="I4" s="10"/>
+    </row>
+    <row r="5" spans="1:9" ht="17" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>20</v>
       </c>
@@ -1015,7 +1054,7 @@
         <v>24</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>24</v>
@@ -1030,10 +1069,10 @@
         <v>1</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="14">
@@ -1044,7 +1083,7 @@
         <v>24</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>24</v>
@@ -1061,24 +1100,24 @@
       <c r="H6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="7"/>
+      <c r="I6" s="10"/>
     </row>
     <row r="7" spans="1:9" ht="14">
       <c r="A7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>1</v>
@@ -1086,7 +1125,7 @@
       <c r="H7" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="7"/>
+      <c r="I7" s="10"/>
     </row>
     <row r="8" spans="1:9" ht="14">
       <c r="A8" s="7" t="s">
@@ -1096,7 +1135,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>25</v>
@@ -1113,7 +1152,7 @@
       <c r="H8" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I8" s="7"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:9" ht="13" customHeight="1">
       <c r="A9" s="7" t="s">
@@ -1123,7 +1162,7 @@
         <v>25</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>25</v>
@@ -1140,7 +1179,7 @@
       <c r="H9" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I9" s="7"/>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:9" ht="13" customHeight="1">
       <c r="A10" s="7" t="s">
@@ -1165,7 +1204,7 @@
       <c r="H10" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="I10" s="7"/>
+      <c r="I10" s="10"/>
     </row>
     <row r="11" spans="1:9" ht="14">
       <c r="A11" s="7" t="s">
@@ -1190,18 +1229,18 @@
       <c r="H11" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I11" s="7"/>
+      <c r="I11" s="10"/>
     </row>
     <row r="12" spans="1:9" ht="14">
       <c r="A12" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>1</v>
@@ -1215,7 +1254,7 @@
       <c r="H12" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I12" s="7"/>
+      <c r="I12" s="10"/>
     </row>
     <row r="13" spans="1:9" ht="14">
       <c r="A13" s="7" t="s">
@@ -1240,7 +1279,7 @@
       <c r="H13" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I13" s="7"/>
+      <c r="I13" s="10"/>
     </row>
     <row r="14" spans="1:9" ht="14">
       <c r="A14" s="7" t="s">
@@ -1265,7 +1304,7 @@
       <c r="H14" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I14" s="7"/>
+      <c r="I14" s="10"/>
     </row>
     <row r="15" spans="1:9" ht="14">
       <c r="A15" s="7" t="s">
@@ -1275,7 +1314,7 @@
         <v>30</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>30</v>
@@ -1292,7 +1331,7 @@
       <c r="H15" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I15" s="7"/>
+      <c r="I15" s="10"/>
     </row>
     <row r="16" spans="1:9" ht="13" customHeight="1">
       <c r="A16" s="7" t="s">
@@ -1302,7 +1341,7 @@
         <v>30</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>30</v>
@@ -1319,7 +1358,7 @@
       <c r="H16" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I16" s="7"/>
+      <c r="I16" s="10"/>
     </row>
     <row r="17" spans="1:9" ht="13" customHeight="1">
       <c r="A17" s="7" t="s">
@@ -1329,7 +1368,7 @@
         <v>31</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>31</v>
@@ -1346,7 +1385,7 @@
       <c r="H17" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I17" s="7"/>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="1:9" ht="13" customHeight="1">
       <c r="A18" s="7" t="s">
@@ -1356,7 +1395,7 @@
         <v>31</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>31</v>
@@ -1373,7 +1412,7 @@
       <c r="H18" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I18" s="7"/>
+      <c r="I18" s="10"/>
     </row>
     <row r="19" spans="1:9" ht="13" customHeight="1">
       <c r="A19" s="7" t="s">
@@ -1383,7 +1422,7 @@
         <v>31</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>31</v>
@@ -1400,7 +1439,7 @@
       <c r="H19" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I19" s="7"/>
+      <c r="I19" s="10"/>
     </row>
     <row r="20" spans="1:9" ht="13" customHeight="1">
       <c r="A20" s="7" t="s">
@@ -1410,7 +1449,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>31</v>
@@ -1427,7 +1466,7 @@
       <c r="H20" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I20" s="7"/>
+      <c r="I20" s="10"/>
     </row>
     <row r="21" spans="1:9" ht="13" customHeight="1">
       <c r="A21" s="7" t="s">
@@ -1437,7 +1476,7 @@
         <v>31</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>31</v>
@@ -1454,7 +1493,7 @@
       <c r="H21" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I21" s="7"/>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" spans="1:9" ht="13" customHeight="1">
       <c r="A22" s="7" t="s">
@@ -1464,7 +1503,7 @@
         <v>31</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>31</v>
@@ -1481,7 +1520,7 @@
       <c r="H22" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I22" s="7"/>
+      <c r="I22" s="10"/>
     </row>
     <row r="23" spans="1:9" ht="13" customHeight="1">
       <c r="A23" s="7" t="s">
@@ -1491,7 +1530,7 @@
         <v>31</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>31</v>
@@ -1509,7 +1548,7 @@
         <v>2</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="13" customHeight="1">
@@ -1535,9 +1574,9 @@
       <c r="H24" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I24" s="7"/>
-    </row>
-    <row r="25" spans="1:9" ht="13" customHeight="1">
+      <c r="I24" s="10"/>
+    </row>
+    <row r="25" spans="1:9" ht="29" customHeight="1">
       <c r="A25" s="7" t="s">
         <v>20</v>
       </c>
@@ -1548,12 +1587,20 @@
       <c r="D25" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="7" t="s">
-        <v>79</v>
+      <c r="E25" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="13" customHeight="1">
@@ -1579,7 +1626,7 @@
       <c r="H26" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I26" s="7"/>
+      <c r="I26" s="10"/>
     </row>
     <row r="27" spans="1:9" ht="13" customHeight="1">
       <c r="A27" s="7" t="s">
@@ -1604,18 +1651,18 @@
       <c r="H27" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I27" s="7"/>
+      <c r="I27" s="10"/>
     </row>
     <row r="28" spans="1:9" ht="13" customHeight="1">
       <c r="A28" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>0</v>
@@ -1629,7 +1676,7 @@
       <c r="H28" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I28" s="7"/>
+      <c r="I28" s="10"/>
     </row>
     <row r="29" spans="1:9" ht="13" customHeight="1">
       <c r="A29" s="7" t="s">
@@ -1639,7 +1686,7 @@
         <v>36</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>36</v>
@@ -1656,7 +1703,7 @@
       <c r="H29" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I29" s="7"/>
+      <c r="I29" s="10"/>
     </row>
     <row r="30" spans="1:9" ht="13" customHeight="1">
       <c r="A30" s="7" t="s">
@@ -1666,7 +1713,7 @@
         <v>36</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>36</v>
@@ -1683,7 +1730,7 @@
       <c r="H30" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I30" s="7"/>
+      <c r="I30" s="10"/>
     </row>
     <row r="31" spans="1:9" ht="13" customHeight="1">
       <c r="A31" s="7" t="s">
@@ -1693,7 +1740,7 @@
         <v>36</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>36</v>
@@ -1710,7 +1757,7 @@
       <c r="H31" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I31" s="7"/>
+      <c r="I31" s="10"/>
     </row>
     <row r="32" spans="1:9" ht="13" customHeight="1">
       <c r="A32" s="7" t="s">
@@ -1720,7 +1767,7 @@
         <v>36</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>36</v>
@@ -1737,35 +1784,35 @@
       <c r="H32" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I32" s="7"/>
+      <c r="I32" s="10"/>
     </row>
     <row r="33" spans="1:9" ht="13" customHeight="1">
       <c r="A33" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>89</v>
+        <v>1</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="14">
@@ -1791,7 +1838,7 @@
       <c r="H34" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I34" s="7"/>
+      <c r="I34" s="10"/>
     </row>
     <row r="35" spans="1:9" ht="13" customHeight="1">
       <c r="A35" s="7" t="s">
@@ -1816,7 +1863,7 @@
       <c r="H35" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I35" s="7"/>
+      <c r="I35" s="10"/>
     </row>
     <row r="36" spans="1:9" ht="13" customHeight="1">
       <c r="A36" s="7" t="s">
@@ -1841,7 +1888,7 @@
       <c r="H36" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I36" s="7"/>
+      <c r="I36" s="10"/>
     </row>
     <row r="37" spans="1:9" ht="13" customHeight="1">
       <c r="A37" s="7" t="s">
@@ -1866,58 +1913,58 @@
       <c r="H37" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I37" s="7"/>
+      <c r="I37" s="10"/>
     </row>
     <row r="38" spans="1:9" ht="13" customHeight="1">
       <c r="A38" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I38" s="7"/>
+        <v>56</v>
+      </c>
+      <c r="I38" s="10"/>
     </row>
     <row r="39" spans="1:9" ht="13" customHeight="1">
       <c r="A39" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>0</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>67</v>
+        <v>61</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="13" customHeight="1">
@@ -1943,7 +1990,7 @@
       <c r="H40" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I40" s="7"/>
+      <c r="I40" s="10"/>
     </row>
     <row r="41" spans="1:9" ht="13" customHeight="1">
       <c r="A41" s="7" t="s">
@@ -1968,7 +2015,7 @@
       <c r="H41" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I41" s="7"/>
+      <c r="I41" s="10"/>
     </row>
     <row r="42" spans="1:9" ht="13" customHeight="1">
       <c r="A42" s="7" t="s">
@@ -1993,7 +2040,7 @@
       <c r="H42" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I42" s="7"/>
+      <c r="I42" s="10"/>
     </row>
     <row r="43" spans="1:9" ht="13" customHeight="1">
       <c r="A43" s="7" t="s">
@@ -2010,8 +2057,8 @@
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
-      <c r="I43" s="7" t="s">
-        <v>79</v>
+      <c r="I43" s="10" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="13" customHeight="1">
@@ -2019,11 +2066,11 @@
         <v>20</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C44" s="6"/>
-      <c r="D44" s="11" t="s">
-        <v>102</v>
+      <c r="D44" s="6" t="s">
+        <v>94</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>1</v>
@@ -2037,17 +2084,17 @@
       <c r="H44" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I44" s="7"/>
-    </row>
-    <row r="45" spans="1:9" ht="13" customHeight="1">
+      <c r="I44" s="10"/>
+    </row>
+    <row r="45" spans="1:9" ht="15" customHeight="1">
       <c r="A45" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>103</v>
+        <v>84</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>95</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>1</v>
@@ -2061,9 +2108,9 @@
       <c r="H45" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I45" s="7"/>
-    </row>
-    <row r="46" spans="1:9" ht="13" customHeight="1">
+      <c r="I45" s="10"/>
+    </row>
+    <row r="46" spans="1:9" ht="33" customHeight="1">
       <c r="A46" s="7" t="s">
         <v>20</v>
       </c>
@@ -2071,51 +2118,55 @@
         <v>45</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D46" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F46" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="I46" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="E46" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G46" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I46" s="7"/>
-    </row>
-    <row r="47" spans="1:9" ht="13" customHeight="1">
-      <c r="A47" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B47" s="6" t="s">
+    </row>
+    <row r="47" spans="1:9" s="12" customFormat="1" ht="42" customHeight="1">
+      <c r="A47" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B47" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C47" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>5</v>
+      <c r="C47" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F47" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H47" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="I47" s="7"/>
+      <c r="H47" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I47" s="15" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="48" spans="1:9" ht="13" customHeight="1">
       <c r="A48" s="7" t="s">
@@ -2125,25 +2176,25 @@
         <v>45</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D48" s="11" t="s">
-        <v>101</v>
+        <v>58</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>61</v>
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="14">
@@ -2154,7 +2205,7 @@
         <v>46</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>46</v>
@@ -2171,7 +2222,7 @@
       <c r="H49" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I49" s="7"/>
+      <c r="I49" s="10"/>
     </row>
     <row r="50" spans="1:9" ht="13" customHeight="1">
       <c r="A50" s="7" t="s">
@@ -2196,32 +2247,32 @@
       <c r="H50" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I50" s="7"/>
+      <c r="I50" s="10"/>
     </row>
     <row r="51" spans="1:9" ht="13" customHeight="1">
       <c r="A51" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C51" s="6"/>
       <c r="D51" s="6" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I51" s="7"/>
+        <v>56</v>
+      </c>
+      <c r="I51" s="10"/>
     </row>
     <row r="52" spans="1:9" ht="13" customHeight="1">
       <c r="A52" s="7" t="s">
@@ -2246,9 +2297,9 @@
       <c r="H52" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I52" s="7"/>
-    </row>
-    <row r="53" spans="1:9" ht="13" customHeight="1">
+      <c r="I52" s="10"/>
+    </row>
+    <row r="53" spans="1:9" ht="31" customHeight="1">
       <c r="A53" s="7" t="s">
         <v>20</v>
       </c>
@@ -2271,7 +2322,9 @@
       <c r="H53" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I53" s="7"/>
+      <c r="I53" s="10" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="54" spans="1:9" ht="13" customHeight="1">
       <c r="A54" s="7" t="s">
@@ -2281,7 +2334,7 @@
         <v>50</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>50</v>
@@ -2298,7 +2351,7 @@
       <c r="H54" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I54" s="7"/>
+      <c r="I54" s="10"/>
     </row>
     <row r="55" spans="1:9" ht="13" customHeight="1">
       <c r="A55" s="7" t="s">
@@ -2308,7 +2361,7 @@
         <v>50</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>50</v>
@@ -2325,7 +2378,7 @@
       <c r="H55" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I55" s="7"/>
+      <c r="I55" s="10"/>
     </row>
     <row r="56" spans="1:9" ht="13" customHeight="1">
       <c r="A56" s="7" t="s">
@@ -2335,7 +2388,7 @@
         <v>50</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>50</v>
@@ -2352,7 +2405,7 @@
       <c r="H56" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="I56" s="7"/>
+      <c r="I56" s="10"/>
     </row>
     <row r="57" spans="1:9" ht="13" customHeight="1">
       <c r="A57" s="7" t="s">
@@ -2377,7 +2430,7 @@
       <c r="H57" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I57" s="7"/>
+      <c r="I57" s="10"/>
     </row>
     <row r="58" spans="1:9" ht="14">
       <c r="B58" s="3"/>
@@ -3796,4 +3849,281 @@
   <pageMargins left="0.74791666666666667" right="0.74791666666666667" top="0.98402777777777772" bottom="0.98402777777777772" header="0.51180555555555551" footer="0.51180555555555551"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="127c0622-349b-4d55-861f-a6e0c5e83458">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACC64E29E39543448BD23604E0AC5C73" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99a0f45d9ee161ee71727cdc03898eea">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="127c0622-349b-4d55-861f-a6e0c5e83458" xmlns:ns3="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="332b75f3650ea407362a692bb0759c94" ns2:_="" ns3:_="">
+    <xsd:import namespace="127c0622-349b-4d55-861f-a6e0c5e83458"/>
+    <xsd:import namespace="8e4324ac-6997-4cf6-a8a2-e55b9409da4b"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="127c0622-349b-4d55-861f-a6e0c5e83458" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8c631306-648b-4820-82d0-96e941587191" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="15" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="21" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{57930aa2-9095-48ab-a7d7-adb860b1acbf}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="8e4324ac-6997-4cf6-a8a2-e55b9409da4b">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CF1D939-3A63-42C4-A733-BED50FF59607}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8e4324ac-6997-4cf6-a8a2-e55b9409da4b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="127c0622-349b-4d55-861f-a6e0c5e83458"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D18150-EF41-4E5C-913E-3061DE707EDA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21AA760D-79DC-4CF4-9298-61452DA0FC23}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="127c0622-349b-4d55-861f-a6e0c5e83458"/>
+    <ds:schemaRef ds:uri="8e4324ac-6997-4cf6-a8a2-e55b9409da4b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Minor edit to headers
</commit_message>
<xml_diff>
--- a/source_data/Ichneumonidae_traits.xlsx
+++ b/source_data/Ichneumonidae_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DFE003E-7008-0F4A-94B8-422EBCEA1F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1945683A-FE16-FE41-BCC3-97D6895F6AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="620" windowWidth="25400" windowHeight="15400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -400,16 +400,16 @@
     <t>Most species are likely associated with hosts on plants; some species are associated with hosts in wood, which may be the ancestral life history</t>
   </si>
   <si>
-    <t>Feeding niche SE</t>
-  </si>
-  <si>
-    <t>Feeding habitat SE</t>
-  </si>
-  <si>
     <t>Feeding niche MG</t>
   </si>
   <si>
     <t>Feeding habitat MG</t>
+  </si>
+  <si>
+    <t>Main feeding niche SE</t>
+  </si>
+  <si>
+    <t>Main feeding habitat SE</t>
   </si>
 </sst>
 </file>
@@ -502,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -524,13 +524,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -862,7 +855,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -906,7 +899,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -956,16 +949,16 @@
         <v>19</v>
       </c>
       <c r="E1" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="I1" s="8" t="s">
         <v>92</v>
@@ -2120,13 +2113,13 @@
       <c r="C46" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E46" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="F46" s="14" t="s">
+      <c r="E46" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="F46" s="11" t="s">
         <v>56</v>
       </c>
       <c r="G46" s="6" t="s">
@@ -2149,22 +2142,22 @@
       <c r="C47" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D47" s="14" t="s">
+      <c r="D47" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E47" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="F47" s="14" t="s">
+      <c r="E47" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="F47" s="11" t="s">
         <v>56</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H47" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="I47" s="15" t="s">
+      <c r="H47" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="I47" s="10" t="s">
         <v>107</v>
       </c>
     </row>
@@ -3852,26 +3845,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="127c0622-349b-4d55-861f-a6e0c5e83458">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACC64E29E39543448BD23604E0AC5C73" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99a0f45d9ee161ee71727cdc03898eea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="127c0622-349b-4d55-861f-a6e0c5e83458" xmlns:ns3="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="332b75f3650ea407362a692bb0759c94" ns2:_="" ns3:_="">
     <xsd:import namespace="127c0622-349b-4d55-861f-a6e0c5e83458"/>
@@ -4084,32 +4057,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CF1D939-3A63-42C4-A733-BED50FF59607}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8e4324ac-6997-4cf6-a8a2-e55b9409da4b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="127c0622-349b-4d55-861f-a6e0c5e83458"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D18150-EF41-4E5C-913E-3061DE707EDA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="127c0622-349b-4d55-861f-a6e0c5e83458">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21AA760D-79DC-4CF4-9298-61452DA0FC23}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4126,4 +4094,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D18150-EF41-4E5C-913E-3061DE707EDA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CF1D939-3A63-42C4-A733-BED50FF59607}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8e4324ac-6997-4cf6-a8a2-e55b9409da4b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="127c0622-349b-4d55-861f-a6e0c5e83458"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Edit of headers for MG data as well
</commit_message>
<xml_diff>
--- a/source_data/Ichneumonidae_traits.xlsx
+++ b/source_data/Ichneumonidae_traits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1945683A-FE16-FE41-BCC3-97D6895F6AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C33039-54D4-184E-A664-1C11F28E321A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="620" windowWidth="25400" windowHeight="15400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -400,16 +400,16 @@
     <t>Most species are likely associated with hosts on plants; some species are associated with hosts in wood, which may be the ancestral life history</t>
   </si>
   <si>
-    <t>Feeding niche MG</t>
-  </si>
-  <si>
-    <t>Feeding habitat MG</t>
-  </si>
-  <si>
     <t>Main feeding niche SE</t>
   </si>
   <si>
     <t>Main feeding habitat SE</t>
+  </si>
+  <si>
+    <t>Main feeding niche MG</t>
+  </si>
+  <si>
+    <t>Main feeding habitat MG</t>
   </si>
 </sst>
 </file>
@@ -855,7 +855,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -899,7 +899,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -949,16 +949,16 @@
         <v>19</v>
       </c>
       <c r="E1" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="I1" s="8" t="s">
         <v>92</v>
@@ -3845,6 +3845,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACC64E29E39543448BD23604E0AC5C73" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99a0f45d9ee161ee71727cdc03898eea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="127c0622-349b-4d55-861f-a6e0c5e83458" xmlns:ns3="8e4324ac-6997-4cf6-a8a2-e55b9409da4b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="332b75f3650ea407362a692bb0759c94" ns2:_="" ns3:_="">
     <xsd:import namespace="127c0622-349b-4d55-861f-a6e0c5e83458"/>
@@ -4057,15 +4066,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4078,6 +4078,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D18150-EF41-4E5C-913E-3061DE707EDA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21AA760D-79DC-4CF4-9298-61452DA0FC23}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4092,14 +4100,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D18150-EF41-4E5C-913E-3061DE707EDA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>